<commit_message>
flexible years; use utac for the join key; output additional columns
</commit_message>
<xml_diff>
--- a/src/make_dummy_data/登録学生一覧.xlsx
+++ b/src/make_dummy_data/登録学生一覧.xlsx
@@ -425,954 +425,2139 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B79"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>共通ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>学籍番号</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>学生氏名</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ごしゅみ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>もくひょー</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>97993510</t>
+          <t>9279013134</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>こーるど ぷれりん</t>
+          <t>98005222</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>なただり りんぴょ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>書店で背表紙を読む</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Gitでやらかさない</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>91159695</t>
+          <t>6169182974</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>にゅとーん いさりん</t>
+          <t>94681791</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>まーく らふりん</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>自販機のラインナップ分析</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>レポートを提出期限より前に出す経験をする</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>90651734</t>
+          <t>3343708628</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ふぇでら ろじゃりん</t>
+          <t>90954705</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>けいと うぃんり</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>レシートの長さランキング</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>深夜のネットサーフィンを控える（理想）</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>91512015</t>
+          <t>0175301378</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ながさま まさみん</t>
+          <t>91820250</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>にしじま ひでとん</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>消しゴムの角を守る</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>今年こそ朝型人間になる（予定）</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>95122801</t>
+          <t>9810224915</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>さかぐてぃ けんたろぴ</t>
+          <t>94287215</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>がりれお るんた</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>新しいショートカットキー探し</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>コーヒーを飲みすぎない</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>94408956</t>
+          <t>9940799401</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>あんどりゅ りんふ</t>
+          <t>98943564</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>にしこり けいたん</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>自販機のラインナップ分析</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>レポートの誤字を減らす</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>98098503</t>
+          <t>4341794494</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>かりすて ふりん</t>
+          <t>96426990</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>でんぜる わしりん</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>雲の形の解釈</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>友達の課題の進み具合を見て焦らない</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>93021805</t>
+          <t>4141435048</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>めしりお ねるん</t>
+          <t>92283434</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>へんりー かびりん</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ペン回し（成功率30%）</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>今年こそ朝型人間になる（予定）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>94011838</t>
+          <t>9130614515</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ひゅー じゃくりん</t>
+          <t>90506589</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>すかーれ っとりん</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Googleマップで遠くの街を散歩</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>講義に出る回数を増やす</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>99072052</t>
+          <t>0127002595</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>える ふぁにんぬ</t>
+          <t>94262459</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>きむたくん たくやん</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>靴ひもを結び直すタイミング研究</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>講義に5分前に着く人になる</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>96123779</t>
+          <t>5001007037</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>まーらー るぴょ</t>
+          <t>96243156</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>よしだ りんちゃ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>天井の模様を眺める</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>研究室の椅子を壊さない</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>90653843</t>
+          <t>0100744423</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>かわぐてぃ はるにゃ</t>
+          <t>94408956</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>あんどりゅ りんふ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>スマホのバッテリー節約術研究</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>レポートの誤字を減らす</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>96716163</t>
+          <t>7612431523</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>りあーな ぴょんぬ</t>
+          <t>97536739</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>さらー りんみゅ</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>コンビニの新商品チェック</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>パスワードを覚えられるものにする</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>90043817</t>
+          <t>9508708530</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>みうらか ずたん</t>
+          <t>93046823</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>きあぬ りぶりん</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>書店で背表紙を読む</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>システムのログインパスワードを忘れない</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>91941830</t>
+          <t>6406409299</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>えどしー らんぴ</t>
+          <t>90722785</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>めしりお ぴょりん</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>レシートの長さランキング</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>スマホを見ない時間を一日5分作る</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>99350122</t>
+          <t>0749763142</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ればんど ふすりん</t>
+          <t>96967984</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>うぃる すみりん</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>コンビニの新商品チェック</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>深夜のネットサーフィンを控える（理想）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>90506589</t>
+          <t>9197188560</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>すかーれ っとりん</t>
+          <t>94504507</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>そんふん みんりん</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>雨が降りそうかどうかの体感予測</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>エレベーターを使わず階段を使う日を作る</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>90954705</t>
+          <t>1840146537</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>けいと うぃんり</t>
+          <t>93251533</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>おおさか なみりん</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>机の上の整理（30分だけ）</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>朝ごはんを食べる日を増やす</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>95012302</t>
+          <t>1003835549</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>えまま そんりん</t>
+          <t>99171192</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ろなくり どるん</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>エスカレーターで立ち位置を考える</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>講義の質問を一度はしてみる</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>91808853</t>
+          <t>5304988098</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>めんでれ ふぃん</t>
+          <t>95556337</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>えじそと とまち</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>スーパーの値引きタイミング観察</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>コーヒーを飲みすぎない</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>90026696</t>
+          <t>5147308611</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>とびー まぐりん</t>
+          <t>94703520</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>えんどう りんみゅ</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>家の周りを一周する</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>研究室の椅子を壊さない</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>94288321</t>
+          <t>3286719596</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ひろしぇ すずたん</t>
+          <t>96195615</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>まついひ できゅ</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>雨が降りそうかどうかの体感予測</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>スマホを見ない時間を一日5分作る</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>90111320</t>
+          <t>1681905967</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>いけえ りかこぴ</t>
+          <t>94011838</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ひゅー じゃくりん</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>早歩きと普通歩きの境界研究</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>パソコンのバックアップを取る</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>91019367</t>
+          <t>6620058677</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>あいしゅ たいんるん</t>
+          <t>90026696</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>とびー まぐりん</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>冷蔵庫の中を定期巡回する</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>課題を提出してから安心して寝る</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>95619961</t>
+          <t>0859912394</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>じぇにふぁ ろれみゅ</t>
+          <t>96503172</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>でぃかぷり おれおん</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>書店で背表紙を読む</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>エレベーターを使わず階段を使う日を作る</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>92833198</t>
+          <t>5691370262</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ろばー とぱりん</t>
+          <t>98098503</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>かりすて ふりん</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>机のガタつき調整</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>講義に5分前に着く人になる</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>96815845</t>
+          <t>3646283907</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>だるびしゅ ゆうにゃ</t>
+          <t>91658723</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>こぺるに くすみゅ</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>コンセントの空きを探す</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>今年こそ朝型人間になる（予定）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>99482770</t>
+          <t>1400073713</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>じょだま いけるん</t>
+          <t>95615247</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>じぇし かちゃり</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>カフェの席取り戦略研究</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>発表スライドを前日に完成させる</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>96471453</t>
+          <t>4451523647</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>はりすた いるんぬ</t>
+          <t>96716163</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>りあーな ぴょんぬ</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>YouTubeおすすめの深掘り</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ノートをちゃんと取る（たぶん）</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>90041840</t>
+          <t>9937157100</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ねいまー るりん</t>
+          <t>92911384</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>とむ ほらりん</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>自販機のラインナップ分析</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>机の上を週に一度は片付ける</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>97526525</t>
+          <t>2871012615</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>きゅりまり りんぬ</t>
+          <t>99422693</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>らべるん みゃ</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>おにぎりの具ランキング更新</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>レポートを提出期限より前に出す経験をする</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>91945063</t>
+          <t>5992764226</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>だにえる くらりん</t>
+          <t>91773905</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>くぼ りんた</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>スマホのホーム画面整理</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>パソコンのアップデートを放置しない</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>96075175</t>
+          <t>7013775407</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>たき りんぴ</t>
+          <t>93222012</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ていすう ふとちゃ</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>新しいボールペンの試し書き</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Wi-Fiが遅いときにまず自分を疑う</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>90514484</t>
+          <t>1718614107</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>みりー ぼびりん</t>
+          <t>93964920</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>えりっく さてぃん</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>メールの件名を考えすぎる</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>課題を提出してから安心して寝る</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>96011456</t>
+          <t>5205327525</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>むばっぺ きゅりん</t>
+          <t>97821911</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>あらがち ゆいりん</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>コーヒーを冷ましすぎる</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>研究室のドアをノックする勇気を持つ</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>98592767</t>
+          <t>9350348454</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>なだる らふぁみゅ</t>
+          <t>93325513</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>おりびあ ころりん</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>消しゴムの角を守る</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>「あとでやる」を減らす</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>91658723</t>
+          <t>5697806189</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>こぺるに くすみゅ</t>
+          <t>97970565</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>はまなべ みなみゅ</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>次にやることを考える</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>USBメモリをなくさない一年にする</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>91142538</t>
+          <t>2728817242</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ありあな ぐらぴょ</t>
+          <t>94602157</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>じぇいく ぎれりん</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>キーボードの掃除（気が向いたとき）</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>レポートを提出期限より前に出す経験をする</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>98536163</t>
+          <t>6392257439</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>よしだま さたろ</t>
+          <t>94072064</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>あでるる ぴょみ</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>スマホのバッテリー節約術研究</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>レポートを提出期限より前に出す経験をする</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>94262459</t>
+          <t>2645754197</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>きむたくん たくやん</t>
+          <t>98574936</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>さんどら ぶるぴ</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>新しいショートカットキー探し</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>スマホを見ない時間を一日5分作る</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>90577055</t>
+          <t>2590396233</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>じぇな おてりん</t>
+          <t>91019367</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>あいしゅ たいんるん</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>天井の模様を眺める</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>パスワードを覚えられるものにする</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>90496767</t>
+          <t>0215274990</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>めりる すとりゃ</t>
+          <t>96471453</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>はりすた いるんぬ</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>カップ麺の待ち時間アレンジ</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>コーヒーを飲みすぎない</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>92983686</t>
+          <t>9877702520</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>えみりー ぶらりん</t>
+          <t>94933437</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>まーご っとりん</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>カレンダーの祝日配置チェック</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>パソコンのアップデートを放置しない</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>97970565</t>
+          <t>4821471876</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>はまなべ みなみゅ</t>
+          <t>92698372</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>もーつぁ るとぴ</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>机のガタつき調整</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>コーヒーを飲みすぎない</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>95615247</t>
+          <t>9478027019</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>じぇし かちゃり</t>
+          <t>90496767</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>めりる すとりゃ</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>スーパーの値引きタイミング観察</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>勉強と休憩のバランスを取る</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>98282607</t>
+          <t>8977460928</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ぶらぴと ぴっとん</t>
+          <t>95012302</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>えまま そんりん</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>電車の発車メロディ研究</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>コーヒーを飲みすぎない</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>96195615</t>
+          <t>2751889001</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>まついひ できゅ</t>
+          <t>90653843</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>かわぐてぃ はるにゃ</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>お菓子のカロリー計算（食べた後）</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>締切という概念と仲良くなる</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>97536739</t>
+          <t>8018780257</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>さらー りんみゅ</t>
+          <t>95768378</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>しょぱん ぴょり</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>近所の猫の行動観察</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>発表スライドを前日に完成させる</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>98496681</t>
+          <t>4357371252</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>はーらん どりん</t>
+          <t>91176779</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>りすとん るみゃ</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>書店で背表紙を読む</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>図書館の静けさに慣れる</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>90228827</t>
+          <t>8224520058</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ぶるーの まるりん</t>
+          <t>91549389</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ぺどり りんぴ</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>スーパーの値引きタイミング観察</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>深夜のネットサーフィンを控える（理想）</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>92698372</t>
+          <t>6480310755</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>もーつぁ るとぴ</t>
+          <t>93746912</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>べん あふりん</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Google検索の予測変換観察</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>パスワードを覚えられるものにする</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>92422894</t>
+          <t>6583911310</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>もりなな ぴょん</t>
+          <t>96011456</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>むばっぺ きゅりん</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>スマホのホーム画面整理</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>今年こそ朝型人間になる（予定）</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>93046823</t>
+          <t>0301866209</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>きあぬ りぶりん</t>
+          <t>90514484</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>みりー ぼびりん</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ペン回し（成功率30%）</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>パスワードを覚えられるものにする</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>95889112</t>
+          <t>5208144369</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>あやせる はるかるん</t>
+          <t>90111320</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>いけえ りかこぴ</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>新しいボールペンの試し書き</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>講義に5分前に着く人になる</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>1973756230</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>98154857</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>ほしのげ げんち</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>早歩きと普通歩きの境界研究</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>寝坊の理由を天候以外にする</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>99704475</t>
+          <t>1301590939</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>けいしー ましゅりん</t>
+          <t>99482770</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>じょだま いけるん</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>おにぎりの具ランキング更新</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>講義に5分前に着く人になる</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>96362653</t>
+          <t>9484049424</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>やまじゃき けんとん</t>
+          <t>98282607</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ぶらぴと ぴっとん</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>コンビニコーヒーの濃さ比較</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>研究室のドアをノックする勇気を持つ</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>93283594</t>
+          <t>3329879191</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>どびゅっし ゅりん</t>
+          <t>94994556</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>きたぐわ けいこちゃ</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>天気予報の答え合わせ</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>研究の進捗を月に一度は作る</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>95848525</t>
+          <t>0892772298</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ふろーれ んすぴ</t>
+          <t>99349852</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>べねでぃ くとりん</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>カップ麺の待ち時間アレンジ</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>締切の前日に焦らない生活を目指す</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>98943564</t>
+          <t>6056625134</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>にしこり けいたん</t>
+          <t>93767436</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ぼるうさ いんたん</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>天井の模様を眺める</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>積読の本を一冊は読む</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>98005222</t>
+          <t>1002495462</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>なただり りんぴょ</t>
+          <t>98916415</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>くりす へむりん</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>電車の吊り広告を全部読む</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ノートをちゃんと取る（たぶん）</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>90302590</t>
+          <t>5397912856</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>すだまちゃ まさきゅ</t>
+          <t>99072052</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>える ふぁにんぬ</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>スーパーの値引きタイミング観察</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>研究の進捗を月に一度は作る</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>99484036</t>
+          <t>7229972588</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>あん ねはさりん</t>
+          <t>97947365</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>ぱすてる るんぴ</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>コンビニコーヒーの濃さ比較</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>USBメモリをなくさない一年にする</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>95809183</t>
+          <t>1318276249</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>たけうてぃ りょうまる</t>
+          <t>97526525</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>きゅりまり りんぬ</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>歩道のタイル模様を追う</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>システムのログインパスワードを忘れない</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>96251330</t>
+          <t>4709001521</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>いにえす たりん</t>
+          <t>91462747</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ふくだん みらきゅ</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>レシートの長さランキング</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>研究室のドアをノックする勇気を持つ</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>98407534</t>
+          <t>4149520758</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ろばーと ぱてりん</t>
+          <t>95122801</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>さかぐてぃ けんたろぴ</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ペットボトルのラベル研究</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>朝ごはんを食べる日を増やす</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>92283434</t>
+          <t>5989834735</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>へんりー かびりん</t>
+          <t>93283594</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>どびゅっし ゅりん</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>YouTubeおすすめの深掘り</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>課題を提出してから安心して寝る</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>90722785</t>
+          <t>5885388060</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>めしりお ぴょりん</t>
+          <t>90302590</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>すだまちゃ まさきゅ</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>雨が降りそうかどうかの体感予測</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>寝坊の理由を天候以外にする</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>92453456</t>
+          <t>1447507810</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>べーとー べんちゃ</t>
+          <t>92422894</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>もりなな ぴょん</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>天井の模様を眺める</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>机の引き出しの化石を整理する</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>90311811</t>
+          <t>1996851040</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>やまだて つとん</t>
+          <t>90919775</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>しょーん めんりん</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>コンビニコーヒーの濃さ比較</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>研究室の椅子を壊さない</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>93633575</t>
+          <t>8272778455</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>おかざき りんぬ</t>
+          <t>95619961</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>じぇにふぁ ろれみゅ</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>書店で背表紙を読む</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>研究室のドアをノックする勇気を持つ</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>91462747</t>
+          <t>3384968416</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ふくだん みらきゅ</t>
+          <t>90041840</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ねいまー るりん</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>雲の形の解釈</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>課題のファイル名をわかりやすくする</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>94287215</t>
+          <t>1694523937</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>がりれお るんた</t>
+          <t>91142538</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ありあな ぐらぴょ</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>スーパーの値引きタイミング観察</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>システムのログインパスワードを忘れない</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>99915396</t>
+          <t>6461961544</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>わおたに しょうたいむ</t>
+          <t>97993510</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>こーるど ぷれりん</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>エアコンの最適温度探し</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>昼夜逆転を月に一度は直す</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>94933437</t>
+          <t>1993810950</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>まーご っとりん</t>
+          <t>96123779</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>まーらー るぴょ</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>コンビニの新商品チェック</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>パソコンのバックアップを取る</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>90339372</t>
+          <t>4662150869</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>てすらん にこぴょ</t>
+          <t>97706335</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ぶらっど ぴょりん</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>キーボードの掃除（気が向いたとき）</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>システムのログインパスワードを忘れない</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>91029201</t>
+          <t>3080831276</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>さかもとは やとりん</t>
+          <t>98536163</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>よしだま さたろ</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>早歩きと普通歩きの境界研究</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>課題を提出してから安心して寝る</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>94944026</t>
+          <t>7846193536</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>くりろな うどりん</t>
+          <t>95571403</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ががれで ぃみゅ</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>メールの件名を考えすぎる</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>システムのログインパスワードを忘れない</t>
         </is>
       </c>
     </row>

</xml_diff>